<commit_message>
dict updates AND fixing search functionality
priority ordering for basic perfect matches in english and basic words in orostara
</commit_message>
<xml_diff>
--- a/files/Oros_Eng_Dictionary.xlsx
+++ b/files/Oros_Eng_Dictionary.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7862" uniqueCount="5359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7863" uniqueCount="5359">
   <si>
     <t xml:space="preserve">Orostara</t>
   </si>
@@ -1123,7 +1123,7 @@
     <t xml:space="preserve">axk</t>
   </si>
   <si>
-    <t xml:space="preserve">with -u ending; literally 'good going/away good' basically; see ‘axren’ for addressing someone you are leaving behind</t>
+    <t xml:space="preserve">with -u ending; literally 'good going’ or 'away good' basically; see ‘axren’ for addressing someone you are leaving behind</t>
   </si>
   <si>
     <t xml:space="preserve">goodbye/bye</t>
@@ -1141,7 +1141,7 @@
     <t xml:space="preserve">axn</t>
   </si>
   <si>
-    <t xml:space="preserve">with -u ending; literally 'good stay/remain good' basically; see ‘axrik’ for addressing someone leaving you</t>
+    <t xml:space="preserve">with -u ending; literally 'good stay’ or 'remain good' basically; see ‘axrik’ for addressing someone leaving you</t>
   </si>
   <si>
     <t xml:space="preserve">ax ren</t>
@@ -3454,7 +3454,7 @@
     <t xml:space="preserve">follow/track</t>
   </si>
   <si>
-    <t xml:space="preserve">clear/trackable/easy to follow</t>
+    <t xml:space="preserve">clear/trackable/easy to follow/straightforward</t>
   </si>
   <si>
     <t xml:space="preserve">camino</t>
@@ -14594,9 +14594,6 @@
     <t xml:space="preserve">my/mine</t>
   </si>
   <si>
-    <t xml:space="preserve">yeh</t>
-  </si>
-  <si>
     <t xml:space="preserve">yah</t>
   </si>
   <si>
@@ -15646,7 +15643,7 @@
     <t xml:space="preserve">xantiy</t>
   </si>
   <si>
-    <t xml:space="preserve">website</t>
+    <t xml:space="preserve">website/application/app/program</t>
   </si>
   <si>
     <t xml:space="preserve">站點</t>
@@ -15721,6 +15718,9 @@
     <t xml:space="preserve">please (request)</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t xml:space="preserve">karipayis</t>
   </si>
   <si>
@@ -16234,25 +16234,7 @@
     <t xml:space="preserve">nasekun</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">for clauses; use </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">'nasek' for single words</t>
-    </r>
+    <t xml:space="preserve">for clauses; use 'nasek' for single words</t>
   </si>
   <si>
     <t xml:space="preserve">nasek hun</t>
@@ -16268,7 +16250,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -16398,12 +16380,6 @@
       <name val="Noto Sans CJK SC"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -40485,59 +40461,59 @@
     </row>
     <row r="955" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A955" s="0" t="s">
+        <v>4823</v>
+      </c>
+      <c r="C955" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D955" s="0" t="s">
         <v>4824</v>
       </c>
-      <c r="C955" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="D955" s="0" t="s">
+      <c r="E955" s="0" t="s">
         <v>4825</v>
       </c>
-      <c r="E955" s="0" t="s">
+      <c r="G955" s="0" t="s">
         <v>4826</v>
-      </c>
-      <c r="G955" s="0" t="s">
-        <v>4827</v>
       </c>
       <c r="M955" s="0" t="s">
         <v>43</v>
       </c>
       <c r="N955" s="0" t="s">
+        <v>4827</v>
+      </c>
+      <c r="O955" s="0" t="s">
+        <v>4823</v>
+      </c>
+      <c r="P955" s="0" t="s">
         <v>4828</v>
-      </c>
-      <c r="O955" s="0" t="s">
-        <v>4824</v>
-      </c>
-      <c r="P955" s="0" t="s">
-        <v>4829</v>
       </c>
     </row>
     <row r="956" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A956" s="0" t="s">
+        <v>4829</v>
+      </c>
+      <c r="D956" s="0" t="s">
         <v>4830</v>
       </c>
-      <c r="D956" s="0" t="s">
+      <c r="H956" s="0" t="s">
         <v>4831</v>
       </c>
-      <c r="H956" s="0" t="s">
+      <c r="M956" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N956" s="0" t="s">
         <v>4832</v>
-      </c>
-      <c r="M956" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N956" s="0" t="s">
-        <v>4833</v>
       </c>
     </row>
     <row r="957" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A957" s="0" t="s">
-        <v>4834</v>
+        <v>4833</v>
       </c>
       <c r="C957" s="0" t="s">
         <v>49</v>
       </c>
       <c r="D957" s="0" t="s">
-        <v>4835</v>
+        <v>4834</v>
       </c>
       <c r="E957" s="0" t="s">
         <v>4026</v>
@@ -40552,38 +40528,38 @@
         <v>0</v>
       </c>
       <c r="N957" s="0" t="s">
+        <v>4835</v>
+      </c>
+      <c r="O957" s="0" t="s">
         <v>4836</v>
-      </c>
-      <c r="O957" s="0" t="s">
-        <v>4837</v>
       </c>
     </row>
     <row r="958" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A958" s="0" t="s">
+        <v>4837</v>
+      </c>
+      <c r="F958" s="0" t="s">
         <v>4838</v>
       </c>
-      <c r="F958" s="0" t="s">
+      <c r="H958" s="0" t="s">
         <v>4839</v>
       </c>
-      <c r="H958" s="0" t="s">
+      <c r="I958" s="0" t="s">
+        <v>4839</v>
+      </c>
+      <c r="M958" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N958" s="0" t="s">
         <v>4840</v>
-      </c>
-      <c r="I958" s="0" t="s">
-        <v>4840</v>
-      </c>
-      <c r="M958" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N958" s="0" t="s">
-        <v>4841</v>
       </c>
     </row>
     <row r="959" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A959" s="0" t="s">
+        <v>4841</v>
+      </c>
+      <c r="B959" s="0" t="s">
         <v>4842</v>
-      </c>
-      <c r="B959" s="0" t="s">
-        <v>4843</v>
       </c>
       <c r="C959" s="0" t="s">
         <v>49</v>
@@ -40592,7 +40568,7 @@
         <v>50</v>
       </c>
       <c r="E959" s="0" t="s">
-        <v>4844</v>
+        <v>4843</v>
       </c>
       <c r="J959" s="0" t="s">
         <v>52</v>
@@ -40601,63 +40577,63 @@
         <v>236</v>
       </c>
       <c r="N959" s="0" t="s">
+        <v>4844</v>
+      </c>
+      <c r="O959" s="0" t="s">
         <v>4845</v>
-      </c>
-      <c r="O959" s="0" t="s">
-        <v>4846</v>
       </c>
     </row>
     <row r="960" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A960" s="0" t="s">
+        <v>4846</v>
+      </c>
+      <c r="D960" s="0" t="s">
         <v>4847</v>
       </c>
-      <c r="D960" s="0" t="s">
+      <c r="E960" s="0" t="s">
         <v>4848</v>
       </c>
-      <c r="E960" s="0" t="s">
+      <c r="M960" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N960" s="0" t="s">
         <v>4849</v>
-      </c>
-      <c r="M960" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N960" s="0" t="s">
-        <v>4850</v>
       </c>
     </row>
     <row r="961" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A961" s="0" t="s">
+        <v>4850</v>
+      </c>
+      <c r="D961" s="0" t="s">
         <v>4851</v>
       </c>
-      <c r="D961" s="0" t="s">
+      <c r="E961" s="0" t="s">
         <v>4852</v>
       </c>
-      <c r="E961" s="0" t="s">
+      <c r="M961" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N961" s="0" t="s">
         <v>4853</v>
-      </c>
-      <c r="M961" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N961" s="0" t="s">
-        <v>4854</v>
       </c>
     </row>
     <row r="962" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A962" s="0" t="s">
+        <v>4854</v>
+      </c>
+      <c r="E962" s="0" t="s">
         <v>4855</v>
       </c>
-      <c r="E962" s="0" t="s">
+      <c r="M962" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N962" s="0" t="s">
         <v>4856</v>
-      </c>
-      <c r="M962" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N962" s="0" t="s">
-        <v>4857</v>
       </c>
     </row>
     <row r="963" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A963" s="0" t="s">
-        <v>4858</v>
+        <v>4857</v>
       </c>
       <c r="C963" s="0" t="s">
         <v>713</v>
@@ -40666,21 +40642,21 @@
         <v>3673</v>
       </c>
       <c r="E963" s="0" t="s">
+        <v>4858</v>
+      </c>
+      <c r="G963" s="0" t="s">
         <v>4859</v>
       </c>
-      <c r="G963" s="0" t="s">
+      <c r="M963" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N963" s="0" t="s">
         <v>4860</v>
-      </c>
-      <c r="M963" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N963" s="0" t="s">
-        <v>4861</v>
       </c>
     </row>
     <row r="964" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A964" s="0" t="s">
-        <v>4862</v>
+        <v>4861</v>
       </c>
       <c r="C964" s="0" t="s">
         <v>49</v>
@@ -40689,7 +40665,7 @@
         <v>148</v>
       </c>
       <c r="E964" s="0" t="s">
-        <v>4863</v>
+        <v>4862</v>
       </c>
       <c r="J964" s="0" t="s">
         <v>150</v>
@@ -40698,27 +40674,27 @@
         <v>32</v>
       </c>
       <c r="N964" s="9" t="s">
+        <v>4863</v>
+      </c>
+      <c r="O964" s="0" t="s">
         <v>4864</v>
       </c>
-      <c r="O964" s="0" t="s">
+      <c r="P964" s="0" t="s">
         <v>4865</v>
-      </c>
-      <c r="P964" s="0" t="s">
-        <v>4866</v>
       </c>
     </row>
     <row r="965" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A965" s="0" t="s">
-        <v>4867</v>
+        <v>4866</v>
       </c>
       <c r="C965" s="0" t="s">
         <v>49</v>
       </c>
       <c r="D965" s="0" t="s">
+        <v>4867</v>
+      </c>
+      <c r="E965" s="0" t="s">
         <v>4868</v>
-      </c>
-      <c r="E965" s="0" t="s">
-        <v>4869</v>
       </c>
       <c r="J965" s="0" t="s">
         <v>74</v>
@@ -40730,47 +40706,47 @@
         <v>0</v>
       </c>
       <c r="N965" s="0" t="s">
-        <v>4870</v>
+        <v>4869</v>
       </c>
     </row>
     <row r="966" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A966" s="0" t="s">
+        <v>4870</v>
+      </c>
+      <c r="C966" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E966" s="0" t="s">
         <v>4871</v>
-      </c>
-      <c r="C966" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E966" s="0" t="s">
-        <v>4872</v>
       </c>
       <c r="M966" s="0" t="s">
         <v>527</v>
       </c>
       <c r="N966" s="9" t="s">
+        <v>4872</v>
+      </c>
+      <c r="O966" s="13" t="s">
         <v>4873</v>
       </c>
-      <c r="O966" s="13" t="s">
+      <c r="P966" s="0" t="s">
         <v>4874</v>
-      </c>
-      <c r="P966" s="0" t="s">
-        <v>4875</v>
       </c>
     </row>
     <row r="967" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A967" s="0" t="s">
+        <v>4875</v>
+      </c>
+      <c r="C967" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E967" s="0" t="s">
         <v>4876</v>
       </c>
-      <c r="C967" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E967" s="0" t="s">
+      <c r="F967" s="0" t="s">
         <v>4877</v>
       </c>
-      <c r="F967" s="0" t="s">
+      <c r="G967" s="0" t="s">
         <v>4878</v>
-      </c>
-      <c r="G967" s="0" t="s">
-        <v>4879</v>
       </c>
       <c r="J967" s="0" t="s">
         <v>667</v>
@@ -40779,27 +40755,27 @@
         <v>32</v>
       </c>
       <c r="N967" s="9" t="s">
+        <v>4879</v>
+      </c>
+      <c r="O967" s="0" t="s">
         <v>4880</v>
       </c>
-      <c r="O967" s="0" t="s">
+      <c r="P967" s="0" t="s">
         <v>4881</v>
-      </c>
-      <c r="P967" s="0" t="s">
-        <v>4882</v>
       </c>
     </row>
     <row r="968" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A968" s="0" t="s">
-        <v>4883</v>
+        <v>4882</v>
       </c>
       <c r="C968" s="0" t="s">
         <v>49</v>
       </c>
       <c r="D968" s="0" t="s">
+        <v>4883</v>
+      </c>
+      <c r="E968" s="0" t="s">
         <v>4884</v>
-      </c>
-      <c r="E968" s="0" t="s">
-        <v>4885</v>
       </c>
       <c r="J968" s="0" t="s">
         <v>74</v>
@@ -40811,44 +40787,44 @@
         <v>0</v>
       </c>
       <c r="N968" s="0" t="s">
-        <v>4886</v>
+        <v>4885</v>
       </c>
     </row>
     <row r="969" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A969" s="0" t="s">
+        <v>4886</v>
+      </c>
+      <c r="C969" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E969" s="0" t="s">
         <v>4887</v>
       </c>
-      <c r="C969" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E969" s="0" t="s">
+      <c r="F969" s="0" t="s">
         <v>4888</v>
-      </c>
-      <c r="F969" s="0" t="s">
-        <v>4889</v>
       </c>
       <c r="M969" s="0" t="s">
         <v>62</v>
       </c>
       <c r="N969" s="0" t="s">
+        <v>4889</v>
+      </c>
+      <c r="P969" s="0" t="s">
         <v>4890</v>
-      </c>
-      <c r="P969" s="0" t="s">
-        <v>4891</v>
       </c>
     </row>
     <row r="970" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A970" s="0" t="s">
+        <v>4891</v>
+      </c>
+      <c r="C970" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E970" s="0" t="s">
         <v>4892</v>
       </c>
-      <c r="C970" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E970" s="0" t="s">
-        <v>4893</v>
-      </c>
       <c r="G970" s="0" t="s">
-        <v>4893</v>
+        <v>4892</v>
       </c>
       <c r="J970" s="0" t="s">
         <v>300</v>
@@ -40860,30 +40836,30 @@
         <v>105</v>
       </c>
       <c r="N970" s="0" t="s">
+        <v>4892</v>
+      </c>
+      <c r="P970" s="0" t="s">
         <v>4893</v>
-      </c>
-      <c r="P970" s="0" t="s">
-        <v>4894</v>
       </c>
     </row>
     <row r="971" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A971" s="0" t="s">
+        <v>4894</v>
+      </c>
+      <c r="C971" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D971" s="4" t="s">
         <v>4895</v>
       </c>
-      <c r="C971" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D971" s="4" t="s">
+      <c r="E971" s="4" t="s">
         <v>4896</v>
       </c>
-      <c r="E971" s="4" t="s">
+      <c r="F971" s="4" t="s">
         <v>4897</v>
       </c>
-      <c r="F971" s="4" t="s">
+      <c r="G971" s="4" t="s">
         <v>4898</v>
-      </c>
-      <c r="G971" s="4" t="s">
-        <v>4899</v>
       </c>
       <c r="K971" s="4"/>
       <c r="L971" s="4"/>
@@ -40891,26 +40867,26 @@
         <v>32</v>
       </c>
       <c r="N971" s="24" t="s">
+        <v>4899</v>
+      </c>
+      <c r="O971" s="6" t="s">
         <v>4900</v>
       </c>
-      <c r="O971" s="6" t="s">
+      <c r="P971" s="6" t="s">
         <v>4901</v>
-      </c>
-      <c r="P971" s="6" t="s">
-        <v>4902</v>
       </c>
     </row>
     <row r="972" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A972" s="0" t="s">
-        <v>4903</v>
+        <v>4902</v>
       </c>
       <c r="C972" s="4"/>
       <c r="D972" s="4" t="s">
-        <v>4904</v>
+        <v>4903</v>
       </c>
       <c r="E972" s="4"/>
       <c r="F972" s="4" t="s">
-        <v>4905</v>
+        <v>4904</v>
       </c>
       <c r="G972" s="4"/>
       <c r="K972" s="4"/>
@@ -40919,67 +40895,67 @@
         <v>0</v>
       </c>
       <c r="N972" s="9" t="s">
-        <v>4906</v>
+        <v>4905</v>
       </c>
       <c r="O972" s="4"/>
       <c r="P972" s="4"/>
     </row>
     <row r="973" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A973" s="0" t="s">
-        <v>4907</v>
+        <v>4906</v>
       </c>
       <c r="C973" s="0" t="s">
         <v>531</v>
       </c>
       <c r="E973" s="0" t="s">
+        <v>4907</v>
+      </c>
+      <c r="F973" s="0" t="s">
         <v>4908</v>
       </c>
-      <c r="F973" s="0" t="s">
+      <c r="G973" s="0" t="s">
         <v>4909</v>
       </c>
-      <c r="G973" s="0" t="s">
+      <c r="I973" s="0" t="s">
         <v>4910</v>
-      </c>
-      <c r="I973" s="0" t="s">
-        <v>4911</v>
       </c>
       <c r="M973" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N973" s="8" t="s">
+        <v>4911</v>
+      </c>
+      <c r="O973" s="6" t="s">
         <v>4912</v>
       </c>
-      <c r="O973" s="6" t="s">
+      <c r="P973" s="6" t="s">
         <v>4913</v>
-      </c>
-      <c r="P973" s="6" t="s">
-        <v>4914</v>
       </c>
     </row>
     <row r="974" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A974" s="0" t="s">
-        <v>4915</v>
+        <v>4914</v>
       </c>
       <c r="C974" s="0" t="s">
         <v>531</v>
       </c>
       <c r="E974" s="0" t="s">
+        <v>4915</v>
+      </c>
+      <c r="F974" s="0" t="s">
         <v>4916</v>
       </c>
-      <c r="F974" s="0" t="s">
+      <c r="G974" s="0" t="s">
         <v>4917</v>
-      </c>
-      <c r="G974" s="0" t="s">
-        <v>4918</v>
       </c>
       <c r="M974" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N974" s="9" t="s">
+        <v>4918</v>
+      </c>
+      <c r="O974" s="6" t="s">
         <v>4919</v>
-      </c>
-      <c r="O974" s="6" t="s">
-        <v>4920</v>
       </c>
       <c r="P974" s="6" t="s">
         <v>968</v>
@@ -40987,30 +40963,30 @@
     </row>
     <row r="975" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A975" s="0" t="s">
+        <v>4920</v>
+      </c>
+      <c r="E975" s="0" t="s">
         <v>4921</v>
       </c>
-      <c r="E975" s="0" t="s">
+      <c r="M975" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N975" s="0" t="s">
         <v>4922</v>
       </c>
-      <c r="M975" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N975" s="0" t="s">
+      <c r="O975" s="0" t="s">
         <v>4923</v>
-      </c>
-      <c r="O975" s="0" t="s">
-        <v>4924</v>
       </c>
     </row>
     <row r="976" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A976" s="0" t="s">
+        <v>4924</v>
+      </c>
+      <c r="C976" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E976" s="0" t="s">
         <v>4925</v>
-      </c>
-      <c r="C976" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E976" s="0" t="s">
-        <v>4926</v>
       </c>
       <c r="J976" s="0" t="s">
         <v>213</v>
@@ -41022,61 +40998,61 @@
         <v>1023</v>
       </c>
       <c r="N976" s="0" t="s">
+        <v>4926</v>
+      </c>
+      <c r="P976" s="0" t="s">
         <v>4927</v>
-      </c>
-      <c r="P976" s="0" t="s">
-        <v>4928</v>
       </c>
     </row>
     <row r="977" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A977" s="0" t="s">
+        <v>4928</v>
+      </c>
+      <c r="E977" s="0" t="s">
         <v>4929</v>
       </c>
-      <c r="E977" s="0" t="s">
+      <c r="M977" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N977" s="0" t="s">
         <v>4930</v>
-      </c>
-      <c r="M977" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N977" s="0" t="s">
-        <v>4931</v>
       </c>
     </row>
     <row r="978" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A978" s="0" t="s">
+        <v>4931</v>
+      </c>
+      <c r="D978" s="0" t="s">
         <v>4932</v>
       </c>
-      <c r="D978" s="0" t="s">
+      <c r="E978" s="0" t="s">
         <v>4933</v>
       </c>
-      <c r="E978" s="0" t="s">
+      <c r="M978" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N978" s="0" t="s">
         <v>4934</v>
-      </c>
-      <c r="M978" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N978" s="0" t="s">
-        <v>4935</v>
       </c>
     </row>
     <row r="979" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A979" s="0" t="s">
+        <v>4935</v>
+      </c>
+      <c r="C979" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E979" s="0" t="s">
         <v>4936</v>
       </c>
-      <c r="C979" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E979" s="0" t="s">
+      <c r="F979" s="0" t="s">
         <v>4937</v>
       </c>
-      <c r="F979" s="0" t="s">
+      <c r="G979" s="0" t="s">
         <v>4938</v>
       </c>
-      <c r="G979" s="0" t="s">
+      <c r="H979" s="0" t="s">
         <v>4939</v>
-      </c>
-      <c r="H979" s="0" t="s">
-        <v>4940</v>
       </c>
       <c r="J979" s="0" t="s">
         <v>144</v>
@@ -41085,27 +41061,27 @@
         <v>32</v>
       </c>
       <c r="N979" s="9" t="s">
+        <v>4940</v>
+      </c>
+      <c r="O979" s="0" t="s">
         <v>4941</v>
       </c>
-      <c r="O979" s="0" t="s">
+      <c r="P979" s="0" t="s">
         <v>4942</v>
-      </c>
-      <c r="P979" s="0" t="s">
-        <v>4943</v>
       </c>
     </row>
     <row r="980" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A980" s="0" t="s">
+        <v>4943</v>
+      </c>
+      <c r="C980" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D980" s="0" t="s">
         <v>4944</v>
       </c>
-      <c r="C980" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="D980" s="0" t="s">
+      <c r="E980" s="0" t="s">
         <v>4945</v>
-      </c>
-      <c r="E980" s="0" t="s">
-        <v>4946</v>
       </c>
       <c r="J980" s="0" t="s">
         <v>213</v>
@@ -41117,21 +41093,21 @@
         <v>43</v>
       </c>
       <c r="N980" s="0" t="s">
+        <v>4946</v>
+      </c>
+      <c r="O980" s="0" t="s">
         <v>4947</v>
       </c>
-      <c r="O980" s="0" t="s">
+      <c r="P980" s="0" t="s">
         <v>4948</v>
-      </c>
-      <c r="P980" s="0" t="s">
-        <v>4949</v>
       </c>
     </row>
     <row r="981" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A981" s="0" t="s">
+        <v>4949</v>
+      </c>
+      <c r="E981" s="0" t="s">
         <v>4950</v>
-      </c>
-      <c r="E981" s="0" t="s">
-        <v>4951</v>
       </c>
       <c r="J981" s="0" t="s">
         <v>213</v>
@@ -41143,24 +41119,24 @@
         <v>0</v>
       </c>
       <c r="N981" s="0" t="s">
+        <v>4951</v>
+      </c>
+      <c r="O981" s="0" t="s">
         <v>4952</v>
-      </c>
-      <c r="O981" s="0" t="s">
-        <v>4953</v>
       </c>
     </row>
     <row r="982" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A982" s="0" t="s">
+        <v>4953</v>
+      </c>
+      <c r="C982" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E982" s="0" t="s">
         <v>4954</v>
       </c>
-      <c r="C982" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E982" s="0" t="s">
+      <c r="F982" s="0" t="s">
         <v>4955</v>
-      </c>
-      <c r="F982" s="0" t="s">
-        <v>4956</v>
       </c>
       <c r="J982" s="0" t="s">
         <v>213</v>
@@ -41172,21 +41148,21 @@
         <v>62</v>
       </c>
       <c r="N982" s="0" t="s">
+        <v>4956</v>
+      </c>
+      <c r="P982" s="0" t="s">
         <v>4957</v>
-      </c>
-      <c r="P982" s="0" t="s">
-        <v>4958</v>
       </c>
     </row>
     <row r="983" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A983" s="0" t="s">
-        <v>4959</v>
+        <v>4958</v>
       </c>
       <c r="C983" s="0" t="s">
         <v>49</v>
       </c>
       <c r="D983" s="0" t="s">
-        <v>4960</v>
+        <v>4959</v>
       </c>
       <c r="E983" s="0" t="s">
         <v>4244</v>
@@ -41201,79 +41177,79 @@
         <v>0</v>
       </c>
       <c r="N983" s="0" t="s">
-        <v>4961</v>
+        <v>4960</v>
       </c>
     </row>
     <row r="984" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A984" s="0" t="s">
+        <v>4961</v>
+      </c>
+      <c r="C984" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D984" s="0" t="s">
         <v>4962</v>
       </c>
-      <c r="C984" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="D984" s="0" t="s">
+      <c r="E984" s="0" t="s">
         <v>4963</v>
       </c>
-      <c r="E984" s="0" t="s">
+      <c r="G984" s="0" t="s">
         <v>4964</v>
-      </c>
-      <c r="G984" s="0" t="s">
-        <v>4965</v>
       </c>
       <c r="M984" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N984" s="9" t="s">
+        <v>4965</v>
+      </c>
+      <c r="O984" s="10" t="s">
         <v>4966</v>
       </c>
-      <c r="O984" s="10" t="s">
+      <c r="P984" s="0" t="s">
         <v>4967</v>
-      </c>
-      <c r="P984" s="0" t="s">
-        <v>4968</v>
       </c>
     </row>
     <row r="985" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A985" s="0" t="s">
+        <v>4968</v>
+      </c>
+      <c r="C985" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E985" s="0" t="s">
         <v>4969</v>
       </c>
-      <c r="C985" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E985" s="0" t="s">
+      <c r="G985" s="0" t="s">
         <v>4970</v>
-      </c>
-      <c r="G985" s="0" t="s">
-        <v>4971</v>
       </c>
       <c r="M985" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N985" s="9" t="s">
+        <v>4971</v>
+      </c>
+      <c r="O985" s="0" t="s">
         <v>4972</v>
       </c>
-      <c r="O985" s="0" t="s">
+      <c r="P985" s="0" t="s">
         <v>4973</v>
-      </c>
-      <c r="P985" s="0" t="s">
-        <v>4974</v>
       </c>
     </row>
     <row r="986" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A986" s="0" t="s">
+        <v>4974</v>
+      </c>
+      <c r="C986" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E986" s="0" t="s">
         <v>4975</v>
       </c>
-      <c r="C986" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E986" s="0" t="s">
+      <c r="F986" s="0" t="s">
         <v>4976</v>
       </c>
-      <c r="F986" s="0" t="s">
+      <c r="G986" s="0" t="s">
         <v>4977</v>
-      </c>
-      <c r="G986" s="0" t="s">
-        <v>4978</v>
       </c>
       <c r="J986" s="0" t="s">
         <v>213</v>
@@ -41282,44 +41258,44 @@
         <v>756</v>
       </c>
       <c r="N986" s="0" t="s">
+        <v>4978</v>
+      </c>
+      <c r="P986" s="0" t="s">
         <v>4979</v>
-      </c>
-      <c r="P986" s="0" t="s">
-        <v>4980</v>
       </c>
     </row>
     <row r="987" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A987" s="0" t="s">
+        <v>4980</v>
+      </c>
+      <c r="C987" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E987" s="0" t="s">
         <v>4981</v>
       </c>
-      <c r="C987" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E987" s="0" t="s">
+      <c r="J987" s="0" t="s">
         <v>4982</v>
-      </c>
-      <c r="J987" s="0" t="s">
-        <v>4983</v>
       </c>
       <c r="M987" s="0" t="s">
         <v>105</v>
       </c>
       <c r="N987" s="0" t="s">
+        <v>4983</v>
+      </c>
+      <c r="P987" s="0" t="s">
         <v>4984</v>
-      </c>
-      <c r="P987" s="0" t="s">
-        <v>4985</v>
       </c>
     </row>
     <row r="988" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A988" s="0" t="s">
+        <v>4985</v>
+      </c>
+      <c r="C988" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E988" s="0" t="s">
         <v>4986</v>
-      </c>
-      <c r="C988" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E988" s="0" t="s">
-        <v>4987</v>
       </c>
       <c r="J988" s="0" t="s">
         <v>74</v>
@@ -41331,18 +41307,18 @@
         <v>1023</v>
       </c>
       <c r="N988" s="0" t="s">
+        <v>4987</v>
+      </c>
+      <c r="P988" s="0" t="s">
         <v>4988</v>
-      </c>
-      <c r="P988" s="0" t="s">
-        <v>4989</v>
       </c>
     </row>
     <row r="989" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A989" s="0" t="s">
+        <v>4989</v>
+      </c>
+      <c r="E989" s="0" t="s">
         <v>4990</v>
-      </c>
-      <c r="E989" s="0" t="s">
-        <v>4991</v>
       </c>
       <c r="J989" s="0" t="s">
         <v>74</v>
@@ -41354,18 +41330,18 @@
         <v>0</v>
       </c>
       <c r="N989" s="0" t="s">
+        <v>4991</v>
+      </c>
+      <c r="O989" s="0" t="s">
         <v>4992</v>
-      </c>
-      <c r="O989" s="0" t="s">
-        <v>4993</v>
       </c>
     </row>
     <row r="990" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A990" s="0" t="s">
+        <v>4993</v>
+      </c>
+      <c r="E990" s="0" t="s">
         <v>4994</v>
-      </c>
-      <c r="E990" s="0" t="s">
-        <v>4995</v>
       </c>
       <c r="J990" s="0" t="s">
         <v>74</v>
@@ -41377,47 +41353,47 @@
         <v>0</v>
       </c>
       <c r="N990" s="0" t="s">
+        <v>4995</v>
+      </c>
+      <c r="O990" s="0" t="s">
         <v>4996</v>
-      </c>
-      <c r="O990" s="0" t="s">
-        <v>4997</v>
       </c>
     </row>
     <row r="991" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A991" s="0" t="s">
+        <v>4997</v>
+      </c>
+      <c r="C991" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E991" s="0" t="s">
         <v>4998</v>
       </c>
-      <c r="C991" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E991" s="0" t="s">
+      <c r="F991" s="0" t="s">
         <v>4999</v>
       </c>
-      <c r="F991" s="0" t="s">
+      <c r="G991" s="0" t="s">
         <v>5000</v>
-      </c>
-      <c r="G991" s="0" t="s">
-        <v>5001</v>
       </c>
       <c r="M991" s="0" t="s">
         <v>105</v>
       </c>
       <c r="N991" s="0" t="s">
+        <v>5001</v>
+      </c>
+      <c r="P991" s="0" t="s">
         <v>5002</v>
-      </c>
-      <c r="P991" s="0" t="s">
-        <v>5003</v>
       </c>
     </row>
     <row r="992" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A992" s="0" t="s">
+        <v>5003</v>
+      </c>
+      <c r="C992" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E992" s="0" t="s">
         <v>5004</v>
-      </c>
-      <c r="C992" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E992" s="0" t="s">
-        <v>5005</v>
       </c>
       <c r="J992" s="0" t="s">
         <v>333</v>
@@ -41426,24 +41402,24 @@
         <v>236</v>
       </c>
       <c r="N992" s="5" t="s">
+        <v>5005</v>
+      </c>
+      <c r="O992" s="6" t="s">
         <v>5006</v>
       </c>
-      <c r="O992" s="6" t="s">
+      <c r="P992" s="6" t="s">
         <v>5007</v>
-      </c>
-      <c r="P992" s="6" t="s">
-        <v>5008</v>
       </c>
     </row>
     <row r="993" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A993" s="0" t="s">
+        <v>5008</v>
+      </c>
+      <c r="C993" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E993" s="0" t="s">
         <v>5009</v>
-      </c>
-      <c r="C993" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E993" s="0" t="s">
-        <v>5010</v>
       </c>
       <c r="J993" s="0" t="s">
         <v>333</v>
@@ -41452,18 +41428,18 @@
         <v>442</v>
       </c>
       <c r="N993" s="0" t="s">
-        <v>5011</v>
+        <v>5010</v>
       </c>
     </row>
     <row r="994" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A994" s="0" t="s">
+        <v>5011</v>
+      </c>
+      <c r="C994" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E994" s="0" t="s">
         <v>5012</v>
-      </c>
-      <c r="C994" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E994" s="0" t="s">
-        <v>5013</v>
       </c>
       <c r="J994" s="0" t="s">
         <v>333</v>
@@ -41472,21 +41448,21 @@
         <v>756</v>
       </c>
       <c r="N994" s="0" t="s">
-        <v>5012</v>
+        <v>5011</v>
       </c>
       <c r="P994" s="6" t="s">
-        <v>5014</v>
+        <v>5013</v>
       </c>
     </row>
     <row r="995" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A995" s="0" t="s">
+        <v>5014</v>
+      </c>
+      <c r="C995" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E995" s="0" t="s">
         <v>5015</v>
-      </c>
-      <c r="C995" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E995" s="0" t="s">
-        <v>5016</v>
       </c>
       <c r="J995" s="0" t="s">
         <v>333</v>
@@ -41495,50 +41471,50 @@
         <v>312</v>
       </c>
       <c r="N995" s="5" t="s">
+        <v>5016</v>
+      </c>
+      <c r="O995" s="6" t="s">
         <v>5017</v>
       </c>
-      <c r="O995" s="6" t="s">
+      <c r="P995" s="6" t="s">
         <v>5018</v>
-      </c>
-      <c r="P995" s="6" t="s">
-        <v>5019</v>
       </c>
     </row>
     <row r="996" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A996" s="0" t="s">
+        <v>5019</v>
+      </c>
+      <c r="C996" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E996" s="0" t="s">
         <v>5020</v>
-      </c>
-      <c r="C996" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E996" s="0" t="s">
-        <v>5021</v>
       </c>
       <c r="J996" s="0" t="s">
         <v>243</v>
       </c>
       <c r="M996" s="0" t="s">
+        <v>5021</v>
+      </c>
+      <c r="N996" s="5" t="s">
         <v>5022</v>
       </c>
-      <c r="N996" s="5" t="s">
+      <c r="O996" s="6" t="s">
         <v>5023</v>
       </c>
-      <c r="O996" s="6" t="s">
+      <c r="P996" s="6" t="s">
         <v>5024</v>
-      </c>
-      <c r="P996" s="6" t="s">
-        <v>5025</v>
       </c>
     </row>
     <row r="997" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A997" s="0" t="s">
+        <v>5025</v>
+      </c>
+      <c r="C997" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E997" s="0" t="s">
         <v>5026</v>
-      </c>
-      <c r="C997" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E997" s="0" t="s">
-        <v>5027</v>
       </c>
       <c r="J997" s="0" t="s">
         <v>333</v>
@@ -41547,24 +41523,24 @@
         <v>32</v>
       </c>
       <c r="N997" s="8" t="s">
+        <v>5027</v>
+      </c>
+      <c r="O997" s="6" t="s">
         <v>5028</v>
       </c>
-      <c r="O997" s="6" t="s">
+      <c r="P997" s="6" t="s">
         <v>5029</v>
-      </c>
-      <c r="P997" s="6" t="s">
-        <v>5030</v>
       </c>
     </row>
     <row r="998" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A998" s="0" t="s">
+        <v>5030</v>
+      </c>
+      <c r="C998" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E998" s="0" t="s">
         <v>5031</v>
-      </c>
-      <c r="C998" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E998" s="0" t="s">
-        <v>5032</v>
       </c>
       <c r="J998" s="0" t="s">
         <v>333</v>
@@ -41573,21 +41549,21 @@
         <v>1023</v>
       </c>
       <c r="N998" s="0" t="s">
+        <v>5032</v>
+      </c>
+      <c r="P998" s="6" t="s">
         <v>5033</v>
-      </c>
-      <c r="P998" s="6" t="s">
-        <v>5034</v>
       </c>
     </row>
     <row r="999" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A999" s="0" t="s">
+        <v>5034</v>
+      </c>
+      <c r="C999" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E999" s="0" t="s">
         <v>5035</v>
-      </c>
-      <c r="C999" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E999" s="0" t="s">
-        <v>5036</v>
       </c>
       <c r="J999" s="0" t="s">
         <v>333</v>
@@ -41596,24 +41572,24 @@
         <v>161</v>
       </c>
       <c r="N999" s="0" t="s">
+        <v>5036</v>
+      </c>
+      <c r="O999" s="6" t="s">
         <v>5037</v>
       </c>
-      <c r="O999" s="6" t="s">
+      <c r="P999" s="6" t="s">
         <v>5038</v>
-      </c>
-      <c r="P999" s="6" t="s">
-        <v>5039</v>
       </c>
     </row>
     <row r="1000" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1000" s="0" t="s">
+        <v>5039</v>
+      </c>
+      <c r="C1000" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1000" s="0" t="s">
         <v>5040</v>
-      </c>
-      <c r="C1000" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1000" s="0" t="s">
-        <v>5041</v>
       </c>
       <c r="J1000" s="0" t="s">
         <v>243</v>
@@ -41622,13 +41598,13 @@
         <v>32</v>
       </c>
       <c r="N1000" s="9" t="s">
+        <v>5041</v>
+      </c>
+      <c r="O1000" s="6" t="s">
         <v>5042</v>
       </c>
-      <c r="O1000" s="6" t="s">
+      <c r="P1000" s="6" t="s">
         <v>5043</v>
-      </c>
-      <c r="P1000" s="6" t="s">
-        <v>5044</v>
       </c>
     </row>
     <row r="1001" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41636,7 +41612,7 @@
         <v>21</v>
       </c>
       <c r="D1001" s="0" t="s">
-        <v>5045</v>
+        <v>5044</v>
       </c>
       <c r="I1001" s="0" t="s">
         <v>16</v>
@@ -41656,16 +41632,16 @@
     </row>
     <row r="1002" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1002" s="0" t="s">
+        <v>5045</v>
+      </c>
+      <c r="B1002" s="0" t="s">
         <v>5046</v>
       </c>
-      <c r="B1002" s="0" t="s">
+      <c r="E1002" s="0" t="s">
         <v>5047</v>
       </c>
-      <c r="E1002" s="0" t="s">
+      <c r="F1002" s="0" t="s">
         <v>5048</v>
-      </c>
-      <c r="F1002" s="0" t="s">
-        <v>5049</v>
       </c>
       <c r="J1002" s="0" t="s">
         <v>213</v>
@@ -41674,18 +41650,18 @@
         <v>0</v>
       </c>
       <c r="N1002" s="0" t="s">
-        <v>5050</v>
+        <v>5049</v>
       </c>
     </row>
     <row r="1003" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1003" s="0" t="s">
+        <v>5050</v>
+      </c>
+      <c r="C1003" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1003" s="0" t="s">
         <v>5051</v>
-      </c>
-      <c r="C1003" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1003" s="0" t="s">
-        <v>5052</v>
       </c>
       <c r="J1003" s="0" t="s">
         <v>243</v>
@@ -41694,30 +41670,30 @@
         <v>32</v>
       </c>
       <c r="N1003" s="9" t="s">
+        <v>5052</v>
+      </c>
+      <c r="O1003" s="6" t="s">
         <v>5053</v>
       </c>
-      <c r="O1003" s="6" t="s">
+      <c r="P1003" s="6" t="s">
         <v>5054</v>
-      </c>
-      <c r="P1003" s="6" t="s">
-        <v>5055</v>
       </c>
     </row>
     <row r="1004" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1004" s="0" t="s">
+        <v>5055</v>
+      </c>
+      <c r="B1004" s="0" t="s">
         <v>5056</v>
       </c>
-      <c r="B1004" s="0" t="s">
+      <c r="C1004" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1004" s="0" t="s">
         <v>5057</v>
       </c>
-      <c r="C1004" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1004" s="0" t="s">
+      <c r="G1004" s="0" t="s">
         <v>5058</v>
-      </c>
-      <c r="G1004" s="0" t="s">
-        <v>5059</v>
       </c>
       <c r="J1004" s="0" t="s">
         <v>243</v>
@@ -41726,161 +41702,161 @@
         <v>32</v>
       </c>
       <c r="N1004" s="9" t="s">
+        <v>5059</v>
+      </c>
+      <c r="O1004" s="6" t="s">
         <v>5060</v>
       </c>
-      <c r="O1004" s="6" t="s">
+      <c r="P1004" s="6" t="s">
         <v>5061</v>
-      </c>
-      <c r="P1004" s="6" t="s">
-        <v>5062</v>
       </c>
     </row>
     <row r="1005" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1005" s="0" t="s">
+        <v>5062</v>
+      </c>
+      <c r="E1005" s="0" t="s">
         <v>5063</v>
       </c>
-      <c r="E1005" s="0" t="s">
+      <c r="F1005" s="0" t="s">
         <v>5064</v>
       </c>
-      <c r="F1005" s="0" t="s">
+      <c r="G1005" s="0" t="s">
         <v>5065</v>
       </c>
-      <c r="G1005" s="0" t="s">
+      <c r="M1005" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1005" s="0" t="s">
         <v>5066</v>
       </c>
-      <c r="M1005" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1005" s="0" t="s">
+      <c r="O1005" s="0" t="s">
         <v>5067</v>
-      </c>
-      <c r="O1005" s="0" t="s">
-        <v>5068</v>
       </c>
     </row>
     <row r="1006" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1006" s="0" t="s">
+        <v>5068</v>
+      </c>
+      <c r="B1006" s="0" t="s">
         <v>5069</v>
       </c>
-      <c r="B1006" s="0" t="s">
+      <c r="D1006" s="0" t="s">
         <v>5070</v>
       </c>
-      <c r="D1006" s="0" t="s">
+      <c r="G1006" s="0" t="s">
         <v>5071</v>
       </c>
-      <c r="G1006" s="0" t="s">
+      <c r="H1006" s="0" t="s">
+        <v>5071</v>
+      </c>
+      <c r="M1006" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1006" s="0" t="s">
         <v>5072</v>
-      </c>
-      <c r="H1006" s="0" t="s">
-        <v>5072</v>
-      </c>
-      <c r="M1006" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1006" s="0" t="s">
-        <v>5073</v>
       </c>
     </row>
     <row r="1007" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1007" s="0" t="s">
+        <v>5073</v>
+      </c>
+      <c r="D1007" s="0" t="s">
         <v>5074</v>
       </c>
-      <c r="D1007" s="0" t="s">
+      <c r="G1007" s="0" t="s">
         <v>5075</v>
       </c>
-      <c r="G1007" s="0" t="s">
+      <c r="H1007" s="0" t="s">
+        <v>5075</v>
+      </c>
+      <c r="M1007" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1007" s="0" t="s">
         <v>5076</v>
-      </c>
-      <c r="H1007" s="0" t="s">
-        <v>5076</v>
-      </c>
-      <c r="M1007" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1007" s="0" t="s">
-        <v>5077</v>
       </c>
     </row>
     <row r="1008" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1008" s="0" t="s">
+        <v>5077</v>
+      </c>
+      <c r="D1008" s="0" t="s">
         <v>5078</v>
       </c>
-      <c r="D1008" s="0" t="s">
+      <c r="G1008" s="0" t="s">
         <v>5079</v>
       </c>
-      <c r="G1008" s="0" t="s">
+      <c r="H1008" s="0" t="s">
+        <v>5079</v>
+      </c>
+      <c r="M1008" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1008" s="0" t="s">
         <v>5080</v>
-      </c>
-      <c r="H1008" s="0" t="s">
-        <v>5080</v>
-      </c>
-      <c r="M1008" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1008" s="0" t="s">
-        <v>5081</v>
       </c>
     </row>
     <row r="1009" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1009" s="0" t="s">
+        <v>5081</v>
+      </c>
+      <c r="D1009" s="0" t="s">
         <v>5082</v>
       </c>
-      <c r="D1009" s="0" t="s">
+      <c r="E1009" s="0" t="s">
         <v>5083</v>
       </c>
-      <c r="E1009" s="0" t="s">
+      <c r="F1009" s="0" t="s">
         <v>5084</v>
       </c>
-      <c r="F1009" s="0" t="s">
+      <c r="M1009" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1009" s="0" t="s">
         <v>5085</v>
-      </c>
-      <c r="M1009" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1009" s="0" t="s">
-        <v>5086</v>
       </c>
     </row>
     <row r="1010" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1010" s="0" t="s">
+        <v>5086</v>
+      </c>
+      <c r="D1010" s="0" t="s">
         <v>5087</v>
       </c>
-      <c r="D1010" s="0" t="s">
+      <c r="E1010" s="0" t="s">
         <v>5088</v>
       </c>
-      <c r="E1010" s="0" t="s">
+      <c r="F1010" s="0" t="s">
+        <v>5084</v>
+      </c>
+      <c r="M1010" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1010" s="0" t="s">
         <v>5089</v>
-      </c>
-      <c r="F1010" s="0" t="s">
-        <v>5085</v>
-      </c>
-      <c r="M1010" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1010" s="0" t="s">
-        <v>5090</v>
       </c>
     </row>
     <row r="1011" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1011" s="0" t="s">
+        <v>5090</v>
+      </c>
+      <c r="F1011" s="0" t="s">
         <v>5091</v>
       </c>
-      <c r="F1011" s="0" t="s">
+      <c r="M1011" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1011" s="0" t="s">
         <v>5092</v>
-      </c>
-      <c r="M1011" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1011" s="0" t="s">
-        <v>5093</v>
       </c>
     </row>
     <row r="1012" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1012" s="0" t="s">
+        <v>5093</v>
+      </c>
+      <c r="F1012" s="0" t="s">
         <v>5094</v>
-      </c>
-      <c r="F1012" s="0" t="s">
-        <v>5095</v>
       </c>
       <c r="M1012" s="0" t="s">
         <v>0</v>
@@ -41891,124 +41867,124 @@
     </row>
     <row r="1013" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1013" s="0" t="s">
+        <v>5095</v>
+      </c>
+      <c r="D1013" s="0" t="s">
         <v>5096</v>
       </c>
-      <c r="D1013" s="0" t="s">
+      <c r="F1013" s="0" t="s">
         <v>5097</v>
       </c>
-      <c r="F1013" s="0" t="s">
+      <c r="M1013" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1013" s="0" t="s">
         <v>5098</v>
-      </c>
-      <c r="M1013" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1013" s="0" t="s">
-        <v>5099</v>
       </c>
     </row>
     <row r="1014" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1014" s="0" t="s">
+        <v>5099</v>
+      </c>
+      <c r="D1014" s="0" t="s">
         <v>5100</v>
       </c>
-      <c r="D1014" s="0" t="s">
+      <c r="F1014" s="0" t="s">
         <v>5101</v>
       </c>
-      <c r="F1014" s="0" t="s">
+      <c r="M1014" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1014" s="0" t="s">
         <v>5102</v>
-      </c>
-      <c r="M1014" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1014" s="0" t="s">
-        <v>5103</v>
       </c>
     </row>
     <row r="1015" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1015" s="0" t="s">
+        <v>5103</v>
+      </c>
+      <c r="D1015" s="0" t="s">
+        <v>5100</v>
+      </c>
+      <c r="F1015" s="0" t="s">
         <v>5104</v>
       </c>
-      <c r="D1015" s="0" t="s">
-        <v>5101</v>
-      </c>
-      <c r="F1015" s="0" t="s">
+      <c r="M1015" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1015" s="0" t="s">
         <v>5105</v>
-      </c>
-      <c r="M1015" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1015" s="0" t="s">
-        <v>5106</v>
       </c>
     </row>
     <row r="1016" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1016" s="0" t="s">
+        <v>5106</v>
+      </c>
+      <c r="D1016" s="0" t="s">
         <v>5107</v>
       </c>
-      <c r="D1016" s="0" t="s">
+      <c r="F1016" s="0" t="s">
         <v>5108</v>
       </c>
-      <c r="F1016" s="0" t="s">
+      <c r="M1016" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1016" s="0" t="s">
         <v>5109</v>
-      </c>
-      <c r="M1016" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1016" s="0" t="s">
-        <v>5110</v>
       </c>
     </row>
     <row r="1017" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1017" s="0" t="s">
+        <v>5110</v>
+      </c>
+      <c r="C1017" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1017" s="0" t="s">
         <v>5111</v>
-      </c>
-      <c r="C1017" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1017" s="0" t="s">
-        <v>5112</v>
       </c>
       <c r="M1017" s="0" t="s">
         <v>312</v>
       </c>
       <c r="N1017" s="0" t="s">
+        <v>5112</v>
+      </c>
+      <c r="O1017" s="6" t="s">
         <v>5113</v>
       </c>
-      <c r="O1017" s="6" t="s">
+      <c r="P1017" s="6" t="s">
         <v>5114</v>
-      </c>
-      <c r="P1017" s="6" t="s">
-        <v>5115</v>
       </c>
     </row>
     <row r="1018" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1018" s="0" t="s">
+        <v>5115</v>
+      </c>
+      <c r="C1018" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1018" s="0" t="s">
         <v>5116</v>
-      </c>
-      <c r="C1018" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1018" s="0" t="s">
-        <v>5117</v>
       </c>
       <c r="M1018" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N1018" s="9" t="s">
+        <v>5117</v>
+      </c>
+      <c r="O1018" s="6" t="s">
         <v>5118</v>
       </c>
-      <c r="O1018" s="6" t="s">
+      <c r="P1018" s="6" t="s">
         <v>5119</v>
-      </c>
-      <c r="P1018" s="6" t="s">
-        <v>5120</v>
       </c>
     </row>
     <row r="1019" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1019" s="0" t="s">
+        <v>5120</v>
+      </c>
+      <c r="E1019" s="0" t="s">
         <v>5121</v>
-      </c>
-      <c r="E1019" s="0" t="s">
-        <v>5122</v>
       </c>
       <c r="J1019" s="0" t="s">
         <v>333</v>
@@ -42017,27 +41993,27 @@
         <v>62</v>
       </c>
       <c r="N1019" s="0" t="s">
+        <v>5122</v>
+      </c>
+      <c r="P1019" s="6" t="s">
         <v>5123</v>
-      </c>
-      <c r="P1019" s="6" t="s">
-        <v>5124</v>
       </c>
     </row>
     <row r="1020" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1020" s="0" t="s">
-        <v>5125</v>
+        <v>5124</v>
       </c>
       <c r="C1020" s="0" t="s">
         <v>713</v>
       </c>
       <c r="D1020" s="0" t="s">
+        <v>5125</v>
+      </c>
+      <c r="E1020" s="0" t="s">
         <v>5126</v>
       </c>
-      <c r="E1020" s="0" t="s">
-        <v>5127</v>
-      </c>
       <c r="F1020" s="0" t="s">
-        <v>5127</v>
+        <v>5126</v>
       </c>
       <c r="M1020" s="0" t="s">
         <v>0</v>
@@ -42048,267 +42024,270 @@
     </row>
     <row r="1021" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1021" s="0" t="s">
-        <v>5128</v>
+        <v>5127</v>
       </c>
       <c r="C1021" s="0" t="s">
         <v>713</v>
       </c>
       <c r="G1021" s="0" t="s">
+        <v>5128</v>
+      </c>
+      <c r="M1021" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1021" s="0" t="s">
         <v>5129</v>
-      </c>
-      <c r="M1021" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1021" s="0" t="s">
-        <v>5130</v>
       </c>
     </row>
     <row r="1022" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1022" s="0" t="s">
+        <v>5130</v>
+      </c>
+      <c r="D1022" s="0" t="s">
         <v>5131</v>
       </c>
-      <c r="D1022" s="0" t="s">
+      <c r="E1022" s="0" t="s">
         <v>5132</v>
       </c>
-      <c r="E1022" s="0" t="s">
+      <c r="M1022" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1022" s="0" t="s">
         <v>5133</v>
-      </c>
-      <c r="M1022" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1022" s="0" t="s">
-        <v>5134</v>
       </c>
     </row>
     <row r="1023" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1023" s="0" t="s">
+        <v>5134</v>
+      </c>
+      <c r="B1023" s="0" t="s">
         <v>5135</v>
-      </c>
-      <c r="B1023" s="0" t="s">
-        <v>5136</v>
       </c>
       <c r="C1023" s="0" t="s">
         <v>49</v>
       </c>
       <c r="E1023" s="0" t="s">
+        <v>5136</v>
+      </c>
+      <c r="M1023" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1023" s="0" t="s">
         <v>5137</v>
-      </c>
-      <c r="M1023" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1023" s="0" t="s">
-        <v>5138</v>
       </c>
     </row>
     <row r="1024" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1024" s="0" t="s">
+        <v>5138</v>
+      </c>
+      <c r="B1024" s="0" t="s">
         <v>5139</v>
-      </c>
-      <c r="B1024" s="0" t="s">
-        <v>5140</v>
       </c>
       <c r="C1024" s="0" t="s">
         <v>49</v>
       </c>
       <c r="D1024" s="0" t="s">
+        <v>5140</v>
+      </c>
+      <c r="E1024" s="0" t="s">
         <v>5141</v>
       </c>
-      <c r="E1024" s="0" t="s">
+      <c r="M1024" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1024" s="0" t="s">
         <v>5142</v>
-      </c>
-      <c r="M1024" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1024" s="0" t="s">
-        <v>5143</v>
       </c>
     </row>
     <row r="1025" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1025" s="0" t="s">
+        <v>5143</v>
+      </c>
+      <c r="B1025" s="0" t="s">
         <v>5144</v>
-      </c>
-      <c r="B1025" s="0" t="s">
-        <v>5145</v>
       </c>
       <c r="C1025" s="0" t="s">
         <v>49</v>
       </c>
       <c r="D1025" s="0" t="s">
-        <v>5141</v>
+        <v>5140</v>
       </c>
       <c r="E1025" s="0" t="s">
+        <v>5145</v>
+      </c>
+      <c r="M1025" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1025" s="0" t="s">
         <v>5146</v>
-      </c>
-      <c r="M1025" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1025" s="0" t="s">
-        <v>5147</v>
       </c>
     </row>
     <row r="1026" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1026" s="0" t="s">
-        <v>5148</v>
+        <v>5147</v>
       </c>
       <c r="C1026" s="0" t="s">
         <v>49</v>
       </c>
       <c r="E1026" s="0" t="s">
+        <v>5148</v>
+      </c>
+      <c r="M1026" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1026" s="0" t="s">
         <v>5149</v>
-      </c>
-      <c r="M1026" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1026" s="0" t="s">
-        <v>5150</v>
       </c>
     </row>
     <row r="1027" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1027" s="0" t="s">
-        <v>5151</v>
+        <v>5150</v>
       </c>
       <c r="C1027" s="0" t="s">
         <v>49</v>
       </c>
       <c r="D1027" s="0" t="s">
+        <v>5151</v>
+      </c>
+      <c r="E1027" s="0" t="s">
         <v>5152</v>
       </c>
-      <c r="E1027" s="0" t="s">
+      <c r="M1027" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1027" s="0" t="s">
         <v>5153</v>
-      </c>
-      <c r="M1027" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1027" s="0" t="s">
-        <v>5154</v>
       </c>
     </row>
     <row r="1028" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1028" s="0" t="s">
-        <v>5155</v>
+        <v>5154</v>
       </c>
       <c r="C1028" s="0" t="s">
         <v>713</v>
       </c>
       <c r="D1028" s="0" t="s">
+        <v>5155</v>
+      </c>
+      <c r="F1028" s="0" t="s">
         <v>5156</v>
       </c>
-      <c r="F1028" s="0" t="s">
+      <c r="M1028" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1028" s="0" t="s">
         <v>5157</v>
-      </c>
-      <c r="M1028" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1028" s="0" t="s">
-        <v>5158</v>
       </c>
     </row>
     <row r="1029" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1029" s="0" t="s">
+        <v>5158</v>
+      </c>
+      <c r="C1029" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1029" s="0" t="s">
         <v>5159</v>
-      </c>
-      <c r="C1029" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1029" s="0" t="s">
-        <v>5160</v>
       </c>
       <c r="M1029" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N1029" s="8" t="s">
+        <v>5160</v>
+      </c>
+      <c r="O1029" s="6" t="s">
         <v>5161</v>
       </c>
-      <c r="O1029" s="6" t="s">
+      <c r="P1029" s="6" t="s">
         <v>5162</v>
-      </c>
-      <c r="P1029" s="6" t="s">
-        <v>5163</v>
       </c>
     </row>
     <row r="1030" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1030" s="0" t="s">
+        <v>5163</v>
+      </c>
+      <c r="B1030" s="0" t="s">
         <v>5164</v>
       </c>
-      <c r="B1030" s="0" t="s">
+      <c r="D1030" s="0" t="s">
         <v>5165</v>
       </c>
-      <c r="D1030" s="0" t="s">
+      <c r="F1030" s="0" t="s">
         <v>5166</v>
       </c>
-      <c r="F1030" s="0" t="s">
+      <c r="M1030" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1030" s="0" t="s">
         <v>5167</v>
-      </c>
-      <c r="M1030" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1030" s="0" t="s">
-        <v>5168</v>
       </c>
     </row>
     <row r="1031" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1031" s="0" t="s">
+        <v>5168</v>
+      </c>
+      <c r="C1031" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1031" s="0" t="s">
         <v>5169</v>
-      </c>
-      <c r="C1031" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1031" s="0" t="s">
-        <v>5170</v>
       </c>
       <c r="M1031" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N1031" s="8" t="s">
+        <v>5170</v>
+      </c>
+      <c r="O1031" s="6" t="s">
         <v>5171</v>
       </c>
-      <c r="O1031" s="6" t="s">
+      <c r="P1031" s="6" t="s">
         <v>5172</v>
-      </c>
-      <c r="P1031" s="6" t="s">
-        <v>5173</v>
       </c>
     </row>
     <row r="1032" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1032" s="0" t="s">
+        <v>5173</v>
+      </c>
+      <c r="B1032" s="0" t="s">
         <v>5174</v>
       </c>
-      <c r="B1032" s="0" t="s">
+      <c r="C1032" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1032" s="0" t="s">
         <v>5175</v>
       </c>
-      <c r="C1032" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1032" s="0" t="s">
+      <c r="F1032" s="0" t="s">
         <v>5176</v>
       </c>
-      <c r="F1032" s="0" t="s">
+      <c r="I1032" s="0" t="s">
         <v>5177</v>
-      </c>
-      <c r="I1032" s="0" t="s">
-        <v>5178</v>
       </c>
       <c r="M1032" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N1032" s="8" t="s">
+        <v>5178</v>
+      </c>
+      <c r="O1032" s="6" t="s">
         <v>5179</v>
       </c>
-      <c r="O1032" s="6" t="s">
+      <c r="P1032" s="6" t="s">
         <v>5180</v>
-      </c>
-      <c r="P1032" s="6" t="s">
-        <v>5181</v>
       </c>
     </row>
     <row r="1033" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1033" s="0" t="s">
+        <v>5181</v>
+      </c>
+      <c r="D1033" s="0" t="s">
         <v>5182</v>
       </c>
-      <c r="D1033" s="0" t="s">
+      <c r="F1033" s="0" t="s">
         <v>5183</v>
       </c>
-      <c r="F1033" s="0" t="s">
+      <c r="I1033" s="0" t="s">
         <v>5184</v>
       </c>
       <c r="M1033" s="0" t="s">
@@ -42326,7 +42305,7 @@
         <v>5186</v>
       </c>
       <c r="F1034" s="0" t="s">
-        <v>5184</v>
+        <v>5183</v>
       </c>
       <c r="M1034" s="0" t="s">
         <v>0</v>
@@ -43060,7 +43039,7 @@
     </row>
     <row r="1083" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1083" s="0" t="s">
-        <v>4847</v>
+        <v>4846</v>
       </c>
       <c r="D1083" s="0" t="s">
         <v>5346</v>
@@ -43072,7 +43051,7 @@
         <v>0</v>
       </c>
       <c r="N1083" s="0" t="s">
-        <v>4850</v>
+        <v>4849</v>
       </c>
     </row>
     <row r="1084" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
blanks break dict display :( also accidently put some stuf in the wrong collumn
</commit_message>
<xml_diff>
--- a/files/Oros_Eng_Dictionary.xlsx
+++ b/files/Oros_Eng_Dictionary.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7865" uniqueCount="5360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7893" uniqueCount="5361">
   <si>
     <t xml:space="preserve">Orostara</t>
   </si>
@@ -16049,6 +16049,9 @@
   </si>
   <si>
     <t xml:space="preserve">Oros sax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEMP</t>
   </si>
   <si>
     <t xml:space="preserve">hacker group on Venus; similar chapter on Mars but I do not remember what it's called</t>
@@ -42808,106 +42811,187 @@
       </c>
     </row>
     <row r="1064" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1064" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1064" s="0" t="s">
+        <v>5296</v>
+      </c>
+      <c r="E1064" s="0" t="s">
+        <v>5297</v>
+      </c>
+      <c r="M1064" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1064" s="0" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="1065" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1065" s="0" t="s">
         <v>5295</v>
       </c>
-      <c r="E1064" s="0" t="s">
-        <v>5296</v>
-      </c>
-    </row>
-    <row r="1065" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D1065" s="0" t="s">
-        <v>5297</v>
+        <v>5298</v>
       </c>
       <c r="E1065" s="0" t="s">
-        <v>5298</v>
+        <v>5299</v>
+      </c>
+      <c r="M1065" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1065" s="0" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="1066" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1066" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1066" s="0" t="s">
-        <v>5299</v>
+        <v>5300</v>
       </c>
       <c r="E1066" s="0" t="s">
-        <v>5300</v>
+        <v>5301</v>
       </c>
       <c r="F1066" s="0" t="s">
-        <v>5301</v>
+        <v>5302</v>
+      </c>
+      <c r="M1066" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1066" s="0" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="1067" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1067" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1067" s="0" t="s">
-        <v>5302</v>
+        <v>5303</v>
       </c>
       <c r="E1067" s="0" t="s">
-        <v>5303</v>
+        <v>5304</v>
+      </c>
+      <c r="M1067" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1067" s="0" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="1068" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1068" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1068" s="0" t="s">
-        <v>5304</v>
+        <v>5305</v>
       </c>
       <c r="E1068" s="0" t="s">
-        <v>5305</v>
+        <v>5306</v>
+      </c>
+      <c r="M1068" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1068" s="0" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="1069" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1069" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1069" s="0" t="s">
-        <v>5306</v>
+        <v>5307</v>
       </c>
       <c r="E1069" s="0" t="s">
         <v>1530</v>
       </c>
+      <c r="M1069" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1069" s="0" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="1070" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1070" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1070" s="0" t="s">
-        <v>5307</v>
+        <v>5308</v>
       </c>
       <c r="E1070" s="0" t="s">
-        <v>5308</v>
+        <v>5309</v>
+      </c>
+      <c r="M1070" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1070" s="0" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="1071" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1071" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1071" s="0" t="s">
-        <v>5309</v>
+        <v>5310</v>
       </c>
       <c r="E1071" s="0" t="s">
-        <v>5310</v>
+        <v>5311</v>
+      </c>
+      <c r="M1071" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1071" s="0" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="1072" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1072" s="0" t="s">
+        <v>5295</v>
+      </c>
       <c r="D1072" s="0" t="s">
-        <v>5311</v>
+        <v>5312</v>
       </c>
       <c r="E1072" s="0" t="s">
-        <v>5312</v>
+        <v>5313</v>
+      </c>
+      <c r="M1072" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="N1072" s="0" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="1073" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1073" s="0" t="s">
-        <v>5313</v>
+        <v>5314</v>
       </c>
       <c r="E1073" s="0" t="s">
-        <v>5314</v>
+        <v>5315</v>
       </c>
       <c r="F1073" s="0" t="s">
-        <v>5315</v>
+        <v>5316</v>
       </c>
       <c r="M1073" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1073" s="0" t="s">
-        <v>5316</v>
+        <v>5317</v>
       </c>
     </row>
     <row r="1074" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1074" s="0" t="s">
-        <v>5317</v>
+        <v>5318</v>
       </c>
       <c r="C1074" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D1074" s="0" t="s">
-        <v>5318</v>
+        <v>5319</v>
       </c>
       <c r="M1074" s="0" t="s">
         <v>0</v>
@@ -42918,75 +43002,75 @@
     </row>
     <row r="1075" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1075" s="0" t="s">
-        <v>5319</v>
+        <v>5320</v>
       </c>
       <c r="G1075" s="0" t="s">
-        <v>5320</v>
+        <v>5321</v>
       </c>
       <c r="M1075" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1075" s="0" t="s">
-        <v>5321</v>
+        <v>5322</v>
       </c>
     </row>
     <row r="1076" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1076" s="0" t="s">
-        <v>5322</v>
+        <v>5323</v>
       </c>
       <c r="E1076" s="0" t="s">
-        <v>5323</v>
+        <v>5324</v>
       </c>
       <c r="M1076" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1076" s="0" t="s">
-        <v>5324</v>
+        <v>5325</v>
       </c>
     </row>
     <row r="1077" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1077" s="0" t="s">
-        <v>5325</v>
+        <v>5326</v>
       </c>
       <c r="I1077" s="0" t="s">
-        <v>5326</v>
+        <v>5327</v>
       </c>
       <c r="M1077" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1077" s="0" t="s">
-        <v>5327</v>
+        <v>5328</v>
       </c>
     </row>
     <row r="1078" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1078" s="0" t="s">
-        <v>5328</v>
+        <v>5329</v>
       </c>
       <c r="B1078" s="0" t="s">
-        <v>5329</v>
+        <v>5330</v>
       </c>
       <c r="D1078" s="0" t="s">
-        <v>5330</v>
+        <v>5331</v>
       </c>
       <c r="G1078" s="0" t="s">
-        <v>5331</v>
+        <v>5332</v>
       </c>
       <c r="M1078" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1078" s="0" t="s">
-        <v>5332</v>
+        <v>5333</v>
       </c>
     </row>
     <row r="1079" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1079" s="0" t="s">
-        <v>5333</v>
+        <v>5334</v>
       </c>
       <c r="C1079" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E1079" s="0" t="s">
-        <v>5334</v>
+        <v>5335</v>
       </c>
       <c r="F1079" s="0" t="s">
         <v>3602</v>
@@ -42995,55 +43079,55 @@
         <v>207</v>
       </c>
       <c r="N1079" s="5" t="s">
-        <v>5335</v>
+        <v>5336</v>
       </c>
       <c r="O1079" s="6" t="s">
-        <v>5336</v>
+        <v>5337</v>
       </c>
       <c r="P1079" s="6" t="s">
-        <v>5337</v>
+        <v>5338</v>
       </c>
     </row>
     <row r="1080" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1080" s="0" t="s">
-        <v>5338</v>
+        <v>5339</v>
       </c>
       <c r="E1080" s="0" t="s">
-        <v>5339</v>
+        <v>5340</v>
       </c>
       <c r="M1080" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1080" s="0" t="s">
-        <v>5340</v>
+        <v>5341</v>
       </c>
     </row>
     <row r="1081" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1081" s="0" t="s">
-        <v>5341</v>
+        <v>5342</v>
       </c>
       <c r="E1081" s="0" t="s">
-        <v>5342</v>
+        <v>5343</v>
       </c>
       <c r="M1081" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1081" s="0" t="s">
-        <v>5343</v>
+        <v>5344</v>
       </c>
     </row>
     <row r="1082" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1082" s="0" t="s">
-        <v>5344</v>
+        <v>5345</v>
       </c>
       <c r="E1082" s="0" t="s">
-        <v>5345</v>
+        <v>5346</v>
       </c>
       <c r="M1082" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1082" s="0" t="s">
-        <v>5346</v>
+        <v>5347</v>
       </c>
     </row>
     <row r="1083" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43051,7 +43135,7 @@
         <v>4846</v>
       </c>
       <c r="D1083" s="0" t="s">
-        <v>5347</v>
+        <v>5348</v>
       </c>
       <c r="E1083" s="0" t="s">
         <v>2817</v>
@@ -43068,7 +43152,7 @@
         <v>4561</v>
       </c>
       <c r="D1084" s="0" t="s">
-        <v>5348</v>
+        <v>5349</v>
       </c>
       <c r="E1084" s="0" t="s">
         <v>2817</v>
@@ -43082,53 +43166,53 @@
     </row>
     <row r="1085" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1085" s="0" t="s">
-        <v>5349</v>
+        <v>5350</v>
       </c>
       <c r="D1085" s="0" t="s">
-        <v>5350</v>
+        <v>5351</v>
       </c>
       <c r="E1085" s="0" t="s">
-        <v>5351</v>
+        <v>5352</v>
       </c>
       <c r="M1085" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1085" s="0" t="s">
-        <v>5352</v>
+        <v>5353</v>
       </c>
     </row>
     <row r="1086" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1086" s="0" t="s">
         <v>2182</v>
       </c>
-      <c r="C1086" s="0" t="s">
-        <v>5353</v>
+      <c r="D1086" s="0" t="s">
+        <v>5354</v>
       </c>
       <c r="I1086" s="0" t="s">
-        <v>5354</v>
+        <v>5355</v>
       </c>
       <c r="M1086" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1086" s="0" t="s">
-        <v>5355</v>
+        <v>5356</v>
       </c>
     </row>
     <row r="1087" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1087" s="0" t="s">
-        <v>5356</v>
-      </c>
-      <c r="C1087" s="0" t="s">
         <v>5357</v>
       </c>
+      <c r="D1087" s="0" t="s">
+        <v>5358</v>
+      </c>
       <c r="I1087" s="0" t="s">
-        <v>5354</v>
+        <v>5355</v>
       </c>
       <c r="M1087" s="0" t="s">
         <v>0</v>
       </c>
       <c r="N1087" s="0" t="s">
-        <v>5358</v>
+        <v>5359</v>
       </c>
     </row>
     <row r="1088" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43136,7 +43220,10 @@
         <v>21</v>
       </c>
       <c r="C1088" s="0" t="s">
-        <v>5359</v>
+        <v>23</v>
+      </c>
+      <c r="D1088" s="0" t="s">
+        <v>5360</v>
       </c>
       <c r="M1088" s="0" t="s">
         <v>0</v>

</xml_diff>